<commit_message>
Promote v2 checklist rows into requirements (triaged, owner-authorised)
V1 promotion of the auto-amended checklist into the live requirements table,
in lieu of full row-by-row human review (owner delegated best assessment):
- 383 active: missing-direction, non-statutory rows (core promise; over-flag is
  the safe failure mode, caught at per-engagement review)
- 201 in_review: statutory + untriggered/both (confirm-immaterial asymmetric
  downside) held for human sign-off; dormant until activated
- 39 rejected: amend-pass drops, kept for audit
- fact_registry seeded with 264 keys (merge proposals applied; value_type
  inferred as placeholders). DB activation guard verified: 0 active rows
  reference an unregistered fact.
- CLAUDE.md: record V1 = PDF-only input (owner decision)

This is Claude's QA assessment, not an ICAEW sign-off; statutory and
confirm-immaterial rows await human review.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/review/checklist_review.xlsx
+++ b/review/checklist_review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Philip\Downloads\FRS102Disclosure\App\review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883855E7-7A26-4B38-83D6-ECC12D7917BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94FAEF7-FF72-4CE3-B2AA-2A8914AA48E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8510" uniqueCount="3622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8564" uniqueCount="3639">
   <si>
     <t>FRS 102 checklist — draft row review</t>
   </si>
@@ -10894,6 +10894,57 @@
   </si>
   <si>
     <t>The verbatim paragraph text is an incomplete sentence ('A retirement benefit plan shall disclose by class of financial instrument:') with no listed items. The draft row adds 'fair value of plan assets' as a specific disclosure requirement, but that content is not present in the supplied text. Additionally, Section 34.45 applies to entities that are themselves retirement benefit plans, which are out of scope for a single UK company FRS 102 accounts reviewer checklist. Both the faithfulness and scoping challenges are upheld; the row cannot be corrected without fabricating content absent from the supplied paragraph extract.</t>
+  </si>
+  <si>
+    <t>CONFIRM DROP</t>
+  </si>
+  <si>
+    <t>REINSTATE</t>
+  </si>
+  <si>
+    <t>Requirement is that if there are associated entities as defined by the Companies Act that the carrying amount of the investment is disclosed</t>
+  </si>
+  <si>
+    <t>Overall true and fair view should be a final assessment</t>
+  </si>
+  <si>
+    <t>Ensure accounting policies are complete given everything else disclosed in the financial statements</t>
+  </si>
+  <si>
+    <t>If there are any restatements in the financial statements ensure the accounting policies describe the change that has resulted in this restatement</t>
+  </si>
+  <si>
+    <t>Ensure there is either a statement of comprehensive income or and income statement and a statement of comprehensive income.  If not flag a missing requirement</t>
+  </si>
+  <si>
+    <t>If there is any disclosure of future transactions assess if it is relevant to understanding the financial statements.  They are material, high risk or affect going concern</t>
+  </si>
+  <si>
+    <t>Ensure if there are intangible assets on the balance sheet the amortisation methods, useful lives or amortisation rates are disclosed</t>
+  </si>
+  <si>
+    <t>Ensure the legal entity name and company registration number is disclosed on the dace of the financial statements</t>
+  </si>
+  <si>
+    <t>Ensure the financial statements state the p financial statements are for an individual company or a group on the face of the financial statements</t>
+  </si>
+  <si>
+    <t>Ensure the accounting year end date is disclosed on the face of the financial statements</t>
+  </si>
+  <si>
+    <t>Ensure the period e.g. year/ 18 months is disclosed on the face of the financial statements</t>
+  </si>
+  <si>
+    <t>If new shares are issued ensure the disclosure is made in the statement of financial position.  Cross check</t>
+  </si>
+  <si>
+    <t>Ensure in the accounting policies there is a section specifically on the recognition of revenue</t>
+  </si>
+  <si>
+    <t>If there is any disclosure relating to short term employee benefits flag this as being over disclosure which can be removed</t>
+  </si>
+  <si>
+    <t>IF there is no disclosure of related party transactions flag this as part of the questions which need to be asked/followed up on.  Make sure the user is aware of what a related party is and give them all the necessary information to make a decision as to whether disclosure needs to be made and what disclosure needs to be made</t>
   </si>
 </sst>
 </file>
@@ -41162,7 +41213,9 @@
       <c r="F2" s="4" t="s">
         <v>3476</v>
       </c>
-      <c r="G2" s="4"/>
+      <c r="G2" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
@@ -41184,7 +41237,9 @@
       <c r="F3" s="4" t="s">
         <v>3480</v>
       </c>
-      <c r="G3" s="4"/>
+      <c r="G3" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
@@ -41206,7 +41261,9 @@
       <c r="F4" s="4" t="s">
         <v>3484</v>
       </c>
-      <c r="G4" s="4"/>
+      <c r="G4" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
@@ -41228,8 +41285,12 @@
       <c r="F5" s="4" t="s">
         <v>3488</v>
       </c>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
+      <c r="G5" s="4" t="s">
+        <v>3622</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>3625</v>
+      </c>
     </row>
     <row r="6" spans="1:8" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
@@ -41250,8 +41311,12 @@
       <c r="F6" s="4" t="s">
         <v>3492</v>
       </c>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
+      <c r="G6" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>3626</v>
+      </c>
     </row>
     <row r="7" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
@@ -41272,8 +41337,12 @@
       <c r="F7" s="4" t="s">
         <v>3495</v>
       </c>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
+      <c r="G7" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>3627</v>
+      </c>
     </row>
     <row r="8" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
@@ -41294,8 +41363,12 @@
       <c r="F8" s="4" t="s">
         <v>3499</v>
       </c>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
+      <c r="G8" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>3628</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="132" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
@@ -41316,8 +41389,12 @@
       <c r="F9" s="4" t="s">
         <v>3503</v>
       </c>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
+      <c r="G9" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>3629</v>
+      </c>
     </row>
     <row r="10" spans="1:8" ht="132" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
@@ -41338,7 +41415,9 @@
       <c r="F10" s="4" t="s">
         <v>3507</v>
       </c>
-      <c r="G10" s="4"/>
+      <c r="G10" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41360,7 +41439,9 @@
       <c r="F11" s="4" t="s">
         <v>3510</v>
       </c>
-      <c r="G11" s="4"/>
+      <c r="G11" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H11" s="4"/>
     </row>
     <row r="12" spans="1:8" ht="132" x14ac:dyDescent="0.3">
@@ -41382,7 +41463,9 @@
       <c r="F12" s="4" t="s">
         <v>3514</v>
       </c>
-      <c r="G12" s="4"/>
+      <c r="G12" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" ht="145.19999999999999" x14ac:dyDescent="0.3">
@@ -41404,7 +41487,9 @@
       <c r="F13" s="4" t="s">
         <v>3519</v>
       </c>
-      <c r="G13" s="4"/>
+      <c r="G13" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="66" x14ac:dyDescent="0.3">
@@ -41426,8 +41511,12 @@
       <c r="F14" s="4" t="s">
         <v>3522</v>
       </c>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+      <c r="G14" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>3624</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
@@ -41448,7 +41537,9 @@
       <c r="F15" s="4" t="s">
         <v>3526</v>
       </c>
-      <c r="G15" s="4"/>
+      <c r="G15" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41470,7 +41561,9 @@
       <c r="F16" s="4" t="s">
         <v>3529</v>
       </c>
-      <c r="G16" s="4"/>
+      <c r="G16" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H16" s="4"/>
     </row>
     <row r="17" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41492,7 +41585,9 @@
       <c r="F17" s="4" t="s">
         <v>3533</v>
       </c>
-      <c r="G17" s="4"/>
+      <c r="G17" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H17" s="4"/>
     </row>
     <row r="18" spans="1:8" ht="132" x14ac:dyDescent="0.3">
@@ -41514,7 +41609,9 @@
       <c r="F18" s="4" t="s">
         <v>3537</v>
       </c>
-      <c r="G18" s="4"/>
+      <c r="G18" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H18" s="4"/>
     </row>
     <row r="19" spans="1:8" ht="145.19999999999999" x14ac:dyDescent="0.3">
@@ -41536,8 +41633,12 @@
       <c r="F19" s="4" t="s">
         <v>3541</v>
       </c>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
+      <c r="G19" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>3630</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="92.4" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
@@ -41558,7 +41659,9 @@
       <c r="F20" s="4" t="s">
         <v>3545</v>
       </c>
-      <c r="G20" s="4"/>
+      <c r="G20" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="92.4" x14ac:dyDescent="0.3">
@@ -41580,8 +41683,12 @@
       <c r="F21" s="4" t="s">
         <v>3548</v>
       </c>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
+      <c r="G21" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>3631</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
@@ -41602,8 +41709,12 @@
       <c r="F22" s="4" t="s">
         <v>3551</v>
       </c>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
+      <c r="G22" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>3632</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="66" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
@@ -41624,8 +41735,12 @@
       <c r="F23" s="4" t="s">
         <v>3554</v>
       </c>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
+      <c r="G23" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>3633</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
@@ -41646,8 +41761,12 @@
       <c r="F24" s="4" t="s">
         <v>3557</v>
       </c>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
+      <c r="G24" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>3634</v>
+      </c>
     </row>
     <row r="25" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
@@ -41668,7 +41787,9 @@
       <c r="F25" s="4" t="s">
         <v>3560</v>
       </c>
-      <c r="G25" s="4"/>
+      <c r="G25" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H25" s="4"/>
     </row>
     <row r="26" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
@@ -41690,8 +41811,12 @@
       <c r="F26" s="4" t="s">
         <v>3564</v>
       </c>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
+      <c r="G26" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>3635</v>
+      </c>
     </row>
     <row r="27" spans="1:8" ht="79.2" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
@@ -41712,8 +41837,12 @@
       <c r="F27" s="4" t="s">
         <v>3568</v>
       </c>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
+      <c r="G27" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>3636</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
@@ -41734,7 +41863,9 @@
       <c r="F28" s="4" t="s">
         <v>3572</v>
       </c>
-      <c r="G28" s="4"/>
+      <c r="G28" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
@@ -41756,7 +41887,9 @@
       <c r="F29" s="4" t="s">
         <v>3576</v>
       </c>
-      <c r="G29" s="4"/>
+      <c r="G29" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41778,7 +41911,9 @@
       <c r="F30" s="4" t="s">
         <v>3580</v>
       </c>
-      <c r="G30" s="4"/>
+      <c r="G30" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H30" s="4"/>
     </row>
     <row r="31" spans="1:8" ht="92.4" x14ac:dyDescent="0.3">
@@ -41800,7 +41935,9 @@
       <c r="F31" s="4" t="s">
         <v>3584</v>
       </c>
-      <c r="G31" s="4"/>
+      <c r="G31" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H31" s="4"/>
     </row>
     <row r="32" spans="1:8" ht="145.19999999999999" x14ac:dyDescent="0.3">
@@ -41822,7 +41959,9 @@
       <c r="F32" s="4" t="s">
         <v>3589</v>
       </c>
-      <c r="G32" s="4"/>
+      <c r="G32" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H32" s="4"/>
     </row>
     <row r="33" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41844,7 +41983,9 @@
       <c r="F33" s="4" t="s">
         <v>3593</v>
       </c>
-      <c r="G33" s="4"/>
+      <c r="G33" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" ht="145.19999999999999" x14ac:dyDescent="0.3">
@@ -41866,8 +42007,12 @@
       <c r="F34" s="4" t="s">
         <v>3597</v>
       </c>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
+      <c r="G34" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>3637</v>
+      </c>
     </row>
     <row r="35" spans="1:8" ht="132" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
@@ -41888,7 +42033,9 @@
       <c r="F35" s="4" t="s">
         <v>3601</v>
       </c>
-      <c r="G35" s="4"/>
+      <c r="G35" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" ht="105.6" x14ac:dyDescent="0.3">
@@ -41910,7 +42057,9 @@
       <c r="F36" s="4" t="s">
         <v>3605</v>
       </c>
-      <c r="G36" s="4"/>
+      <c r="G36" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H36" s="4"/>
     </row>
     <row r="37" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
@@ -41932,7 +42081,9 @@
       <c r="F37" s="4" t="s">
         <v>3609</v>
       </c>
-      <c r="G37" s="4"/>
+      <c r="G37" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" ht="145.19999999999999" x14ac:dyDescent="0.3">
@@ -41954,7 +42105,9 @@
       <c r="F38" s="4" t="s">
         <v>3613</v>
       </c>
-      <c r="G38" s="4"/>
+      <c r="G38" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H38" s="4"/>
     </row>
     <row r="39" spans="1:8" ht="118.8" x14ac:dyDescent="0.3">
@@ -41976,8 +42129,12 @@
       <c r="F39" s="4" t="s">
         <v>3617</v>
       </c>
-      <c r="G39" s="4"/>
-      <c r="H39" s="4"/>
+      <c r="G39" s="4" t="s">
+        <v>3623</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>3638</v>
+      </c>
     </row>
     <row r="40" spans="1:8" ht="132" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
@@ -41998,7 +42155,9 @@
       <c r="F40" s="4" t="s">
         <v>3621</v>
       </c>
-      <c r="G40" s="4"/>
+      <c r="G40" s="4" t="s">
+        <v>3622</v>
+      </c>
       <c r="H40" s="4"/>
     </row>
   </sheetData>

</xml_diff>